<commit_message>
Revise outlets 13-20 cost from RM250k to RM450k
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YagSmcBjM8HgRiPUW2dW7u
</commit_message>
<xml_diff>
--- a/output/Outlet_Payment_Timeline_2026.xlsx
+++ b/output/Outlet_Payment_Timeline_2026.xlsx
@@ -796,7 +796,7 @@
         <v>46342</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>250000</v>
+        <v>450000</v>
       </c>
       <c r="E10" s="8" t="n">
         <v>0</v>
@@ -837,7 +837,7 @@
         <v>46344</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>250000</v>
+        <v>450000</v>
       </c>
       <c r="E11" s="8" t="n">
         <v>0</v>
@@ -878,7 +878,7 @@
         <v>46344</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>250000</v>
+        <v>450000</v>
       </c>
       <c r="E12" s="8" t="n">
         <v>0</v>
@@ -919,7 +919,7 @@
         <v>46349</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>250000</v>
+        <v>450000</v>
       </c>
       <c r="E13" s="8" t="n">
         <v>0</v>
@@ -960,7 +960,7 @@
         <v>46356</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>250000</v>
+        <v>450000</v>
       </c>
       <c r="E14" s="8" t="n">
         <v>0</v>
@@ -1001,7 +1001,7 @@
         <v>46363</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>250000</v>
+        <v>450000</v>
       </c>
       <c r="E15" s="8" t="n">
         <v>0</v>
@@ -1042,7 +1042,7 @@
         <v>46365</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>250000</v>
+        <v>450000</v>
       </c>
       <c r="E16" s="8" t="n">
         <v>0</v>
@@ -1083,7 +1083,7 @@
         <v>46371</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>250000</v>
+        <v>450000</v>
       </c>
       <c r="E17" s="8" t="n">
         <v>0</v>
@@ -1133,14 +1133,14 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Not included: #21 ICOMSRWK (grand opening TBD) – add a row when the date is confirmed (RM250,000).</t>
+          <t>Not included: #21 ICOMSRWK (grand opening TBD) – add a row when the date is confirmed (RM450,000).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Source: grand opening dates, costs (RM650k for #10–12, RM250k for #13–20) and amounts paid to Sep were provided by the user.</t>
+          <t>Source: grand opening dates, costs (RM650k for #10–12, RM450k for #13–20) and amounts paid to Sep were provided by the user.</t>
         </is>
       </c>
     </row>

</xml_diff>